<commit_message>
modified:   clauseguard/api/review.py 	modified:   frontend/src/pages/ContractDetail.tsx 	modified:   frontend/src/pages/Review.tsx 	modified:   sample_review_export.xlsx
</commit_message>
<xml_diff>
--- a/sample_review_export.xlsx
+++ b/sample_review_export.xlsx
@@ -79,12 +79,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -540,7 +540,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-09T11:50:54.073040+00:00</t>
+          <t>2026-06-10T07:40:05.149138+00:00</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -596,12 +596,12 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Confidentiality obligations must be defined and enforced.</t>
+          <t>sec. Confidentiality · clause 1.3</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>The agreement includes clear confidentiality obligations that both parties must adhere to.</t>
+          <t>The confidentiality obligations survive for two years after termination, which is a reasonable duration.</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Confidentiality obligations must be defined and enforced.</t>
+          <t>Confidentiality obligations must survive termination for a reasonable period.</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -628,12 +628,12 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Indemnification clauses must be present.</t>
+          <t>sec. Data Protection · clause 6.1</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>The agreement includes an indemnification clause that protects both parties.</t>
+          <t>The agreement states that both parties shall implement reasonable security measures to protect personal data.</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Indemnification clauses must be present.</t>
+          <t>Parties must implement reasonable security measures for data protection.</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -660,12 +660,12 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Limitation of liability must be defined.</t>
+          <t>sec. Termination · clause 5.1</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>The agreement specifies a limitation of liability for both parties.</t>
+          <t>The agreement specifies that upon termination, each party shall return or destroy all Confidential Information.</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Limitation of liability must be defined.</t>
+          <t>The agreement must specify the return or destruction of Confidential Information upon termination.</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -692,44 +692,44 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Governing law must be specified.</t>
+          <t>sec. General Provisions · clause 7.1</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>The agreement specifies that it is governed by the laws of California.</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>low</t>
+          <t>The agreement does not include any provisions for audit rights, which are essential for ensuring compliance with confidentiality and data protection obligations.</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Governing law must be specified.</t>
+          <t>The agreement must include audit rights to ensure compliance.</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>No remediation needed as the requirement is met.</t>
+          <t>Add a clause that grants audit rights to ensure compliance with confidentiality and data protection obligations.</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>No remediation needed as the requirement is met.</t>
+          <t>Add a clause that grants audit rights to ensure compliance with confidentiality and data protection obligations.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Termination clauses must be included.</t>
+          <t>sec. Data Protection · clause 6.1</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>The agreement includes a termination clause allowing either party to terminate with notice.</t>
+          <t>The agreement states that both parties shall comply with applicable data protection laws.</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Termination clauses must be included.</t>
+          <t>The agreement must comply with applicable data protection laws.</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -756,704 +756,544 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Data protection compliance must be addressed.</t>
+          <t>sec. Section 1. Confidentiality · clause 1.3</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>The agreement includes a clause requiring compliance with applicable data protection laws.</t>
+          <t>The confidentiality obligations only survive for two years after termination, which may not be sufficient for certain sensitive information.</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Data protection compliance must be addressed.</t>
+          <t>Duration of confidentiality obligations</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>No remediation needed as the requirement is met.</t>
+          <t>Extend the duration of confidentiality obligations to a longer period, such as five years or indefinitely for certain types of information.</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>No remediation needed as the requirement is met.</t>
+          <t>The confidentiality obligations shall survive for a period of five (5) years after the termination of this Agreement, or indefinitely for trade secrets.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Audit rights must be included.</t>
+          <t>sec. Section 3. Limitation of Liability · clause 3.1</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>The agreement does not include any provisions for audit rights.</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
+          <t>The limitation of liability clause does not account for liabilities arising from gross negligence or willful misconduct, which should be excluded from any cap on liability.</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Audit rights must be included.</t>
+          <t>Limitation of liability for gross negligence or willful misconduct</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Include a clause that grants audit rights to ensure compliance with the agreement.</t>
+          <t>Specify that the limitation of liability does not apply to damages resulting from gross negligence or willful misconduct.</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Include a clause that grants audit rights to ensure compliance with the agreement.</t>
+          <t>Notwithstanding the limitation of liability set forth in this Agreement, neither party shall be liable for any damages arising from its gross negligence or willful misconduct.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Duration of confidentiality obligations</t>
+          <t>sec. Section 5. Termination · clause 5.1</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>The confidentiality obligations only survive for two years after termination, which may not be sufficient for certain types of sensitive information.</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
+          <t>The current clause does not specify a timeline for the return or destruction of Confidential Information after termination.</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Duration of confidentiality obligations</t>
+          <t>Return or destruction of Confidential Information upon termination</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Extend the duration of confidentiality obligations to a longer period or make them indefinite for certain types of sensitive information.</t>
+          <t>Include a specific timeframe within which Confidential Information must be returned or destroyed after termination.</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>The confidentiality obligations shall survive for a period of five (5) years after the termination of this Agreement, or indefinitely for trade secrets and other highly sensitive information.</t>
+          <t>Upon termination, each party shall return or destroy all Confidential Information received from the other party within thirty (30) days.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Limitation of liability for indemnification</t>
+          <t>sec. Section 4. Governing Law · clause 4.1</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>The indemnification clause does not specify any limitations on liability, which could expose parties to significant financial risk.</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
+          <t>The agreement does not specify a process for dispute resolution, such as mediation or arbitration, which could help resolve conflicts more efficiently.</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Limitation of liability for indemnification</t>
+          <t>Dispute resolution mechanism</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Introduce a cap on indemnification liability to provide a clear limit on potential exposure.</t>
+          <t>Incorporate a clause that outlines a preferred dispute resolution process, such as mediation followed by arbitration.</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>The total liability of either party under this indemnification provision shall not exceed the total fees paid under this Agreement or $50,000, whichever is greater.</t>
+          <t>In the event of any dispute arising out of or related to this Agreement, the parties agree to first attempt to resolve the dispute through mediation. If mediation is unsuccessful, the dispute shall be resolved by binding arbitration in accordance with the rules of the American Arbitration Association.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Dispute resolution process</t>
+          <t>sec. Section 1. Confidentiality · clause 1.2</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>The agreement only mentions jurisdiction but lacks a detailed dispute resolution process, such as mediation or arbitration.</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
+          <t>Potential unauthorized disclosure of Confidential Information</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Dispute resolution process</t>
+          <t>Confidentiality</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Incorporate a multi-step dispute resolution process that includes negotiation, mediation, and arbitration before litigation.</t>
+          <t>Implement strict access controls and training for employees on confidentiality obligations.</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>In the event of a dispute, the Parties agree to first attempt to resolve the dispute through good faith negotiation. If unresolved, the Parties shall proceed to mediation, and if still unresolved, to binding arbitration in accordance with the rules of the American Arbitration Association.</t>
+          <t>Implement strict access controls and training for employees on confidentiality obligations.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Data breach notification</t>
+          <t>sec. Section 3. Limitation of Liability · clause 3.1</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>The agreement lacks a clause requiring notification in the event of a data breach involving Confidential Information.</t>
+          <t>Limited liability for breaches may not cover all damages</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Data breach notification</t>
+          <t>Indemnification</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Add a clause that mandates prompt notification of any data breaches affecting Confidential Information.</t>
+          <t>Consider negotiating higher liability limits or removing the limitation clause for certain types of breaches.</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>In the event of a data breach involving Confidential Information, the affected party shall notify the other party within 72 hours of becoming aware of the breach.</t>
+          <t>Consider negotiating higher liability limits or removing the limitation clause for certain types of breaches.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Confidentiality</t>
+          <t>sec. Section 6. Data Protection · clause 6.1</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Potential unauthorized disclosure of Confidential Information</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="inlineStr">
+          <t>Non-compliance with data protection laws</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Confidentiality</t>
+          <t>Data Protection</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Implement strict access controls and regular training on confidentiality obligations for employees.</t>
+          <t>Conduct regular audits and ensure both parties are aware of and comply with relevant data protection regulations.</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Implement strict access controls and regular training on confidentiality obligations for employees.</t>
+          <t>Conduct regular audits and ensure both parties are aware of and comply with relevant data protection regulations.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Indemnification</t>
+          <t>sec. Section 5. Termination · clause 5.1</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Insufficient indemnification clauses</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
+          <t>Unilateral termination may disrupt business operations</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Indemnification</t>
+          <t>Termination</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Review and expand the indemnification clause to cover a broader range of liabilities and ensure clarity.</t>
+          <t>Negotiate longer notice periods or conditions for termination to minimize disruption.</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Review and expand the indemnification clause to cover a broader range of liabilities and ensure clarity.</t>
+          <t>Negotiate longer notice periods or conditions for termination to minimize disruption.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Limitation of Liability</t>
+          <t>sec. Section 1. Confidentiality · clause 1.1</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Cap on liability may be too low</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="inlineStr">
+          <t>Parties must keep all confidential information received from each other private.</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Limitation of Liability</t>
+          <t>Confidentiality</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Consider negotiating a higher liability cap based on the potential risks involved in the business relationship.</t>
+          <t>Potential exposure to loss of proprietary information if confidentiality is breached.</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Consider negotiating a higher liability cap based on the potential risks involved in the business relationship.</t>
+          <t>Ensure all employees are trained on confidentiality obligations.; Implement strict access controls to confidential information.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Governing Law</t>
+          <t>sec. Section 2. Indemnification · clause 2.1</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Jurisdiction limitations</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>low</t>
+          <t>Parties agree to indemnify each other for breaches of the Agreement.</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Governing Law</t>
+          <t>Indemnity</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Negotiate a more neutral jurisdiction or allow for arbitration as an alternative dispute resolution method.</t>
+          <t>Significant financial liability if a breach occurs.</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Negotiate a more neutral jurisdiction or allow for arbitration as an alternative dispute resolution method.</t>
+          <t>Review indemnification clauses regularly to ensure they are adequate.; Consider obtaining insurance to cover potential indemnity claims.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Data Protection</t>
+          <t>sec. Section 3. Limitation of Liability · clause 3.1</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Non-compliance with data protection laws</t>
+          <t>Limits the liability of each party to $50,000 and excludes certain types of damages.</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Data Protection</t>
+          <t>Liability</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Conduct regular audits and ensure both parties have robust data protection policies in place.</t>
+          <t>Limits recovery in case of significant losses.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Conduct regular audits and ensure both parties have robust data protection policies in place.</t>
+          <t>Evaluate whether the liability cap is sufficient for your business needs.; Consider negotiating higher liability limits if necessary.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Confidentiality</t>
+          <t>sec. Section 5. Termination · clause 5.1</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Obligates both parties to keep shared confidential information private.</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
+          <t>Allows either party to terminate the Agreement with notice and requires return of confidential information.</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>confidentiality</t>
+          <t>Termination</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Protects sensitive information from unauthorized disclosure.</t>
+          <t>Provides an exit strategy but requires careful handling of confidential information.</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Ensure all employees are trained on confidentiality obligations.; Regularly review and update confidentiality practices.</t>
+          <t>Establish a clear process for returning or destroying confidential information upon termination.; Ensure all parties are aware of termination procedures.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Indemnification</t>
+          <t>sec. Section 6. Data Protection · clause 6.1</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Provides for indemnification between the parties for breaches of the agreement.</t>
-        </is>
-      </c>
-      <c r="C26" s="11" t="inlineStr">
+          <t>Parties must adhere to data protection laws and implement security measures for personal data.</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>indemnity</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Potential financial liability for breaches could be significant.</t>
+          <t>Non-compliance could lead to legal penalties and reputational damage.</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Consider obtaining insurance to cover potential indemnity claims.; Review indemnity provisions regularly to ensure adequacy.</t>
+          <t>Conduct regular audits to ensure compliance with data protection laws.; Implement robust data security measures and training for employees.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Limitation of Liability</t>
+          <t>sec. Section 4. Governing Law · clause 4.1</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Limits the liability of both parties to direct damages up to $50,000.</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
+          <t>Specifies California law as governing and San Francisco courts for dispute resolution.</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>liability</t>
+          <t>Dispute Resolution</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Limits financial exposure but may not cover all potential damages.</t>
+          <t>Determines the legal framework and jurisdiction for disputes.</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Evaluate whether the liability cap is sufficient for your business.; Consider negotiating higher liability limits if necessary.</t>
+          <t>Consider the implications of jurisdiction on potential disputes.; Ensure legal representation is familiar with California law.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Termination</t>
+          <t>sec. Section 1. Confidentiality · clause 1.3</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Allows either party to terminate the agreement with notice.</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>low</t>
+          <t>Extending the confidentiality period protects sensitive information for a longer duration, which is crucial for business interests.</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>termination</t>
+          <t>Extend the confidentiality obligations beyond two years.</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Provides flexibility to exit the agreement but requires notice.</t>
+          <t>These confidentiality obligations shall survive for a period of five (5) years after the termination of this Agreement.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Ensure proper procedures are in place for termination.; Maintain records of all confidential information for compliance.</t>
+          <t>These confidentiality obligations shall survive for a period of five (5) years after the termination of this Agreement.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Data Protection</t>
+          <t>sec. Section 3. Limitation of Liability · clause 3.1</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Mandates compliance with data protection laws and security measures.</t>
+          <t>This change ensures that parties are only liable for direct damages, reducing the risk of unforeseen financial exposure.</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>privacy</t>
+          <t>Limit liability to direct damages only.</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Failure to comply could result in legal penalties.</t>
+          <t>The total liability of either party shall not exceed the amount of direct damages incurred, up to fifty thousand dollars ($50,000).</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Conduct regular audits of data protection practices.; Stay updated on changes in data protection laws.</t>
+          <t>The total liability of either party shall not exceed the amount of direct damages incurred, up to fifty thousand dollars ($50,000).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>Governing Law and Dispute Resolution</t>
+          <t>sec. Section 5. Termination · clause 5.1</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Establishes California law as governing and specifies dispute resolution location.</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="inlineStr">
+          <t>Adding a confirmation requirement ensures accountability and provides a clear record of compliance with the confidentiality obligations.</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>dispute resolution</t>
+          <t>Clarify the process for returning or destroying Confidential Information.</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Determines legal jurisdiction for any disputes.</t>
+          <t>Upon termination, each party shall return or destroy all Confidential Information received from the other party, and provide written confirmation of such return or destruction.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Consider the implications of California law on your business.; Prepare for potential disputes in the specified jurisdiction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>Extend the confidentiality obligations beyond two years.</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Extending the confidentiality period protects both parties' sensitive information for a longer duration, which is crucial in competitive industries.</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>Extend the confidentiality obligations beyond two years.</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>These confidentiality obligations shall survive for a period of five (5) years after the termination of this Agreement.</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>These confidentiality obligations shall survive for a period of five (5) years after the termination of this Agreement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>Clarify the definition of Confidential Information.</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>This clarification ensures both parties have a mutual understanding of what information is protected, reducing the risk of inadvertent disclosures.</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>Clarify the definition of Confidential Information.</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>Confidential Information shall also include any information that is marked as confidential or that is disclosed in a manner that indicates its confidential nature.</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="inlineStr">
-        <is>
-          <t>Confidential Information shall also include any information that is marked as confidential or that is disclosed in a manner that indicates its confidential nature.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>Limit the indemnification clause to direct damages only.</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>This change minimizes the financial risk for both parties and aligns with standard industry practices.</t>
-        </is>
-      </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>Limit the indemnification clause to direct damages only.</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>Each party shall indemnify and hold harmless the other party from and against any direct claims, damages, and losses arising out of a breach of this Agreement by the indemnifying party.</t>
-        </is>
-      </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>Each party shall indemnify and hold harmless the other party from and against any direct claims, damages, and losses arising out of a breach of this Agreement by the indemnifying party.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>Modify the limitation of liability clause to include a cap on indirect damages.</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>This ensures that both parties are protected from excessive liability while still holding them accountable for serious breaches.</t>
-        </is>
-      </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>Modify the limitation of liability clause to include a cap on indirect damages.</t>
-        </is>
-      </c>
-      <c r="E34" s="9" t="inlineStr">
-        <is>
-          <t>Neither party shall be liable for any indirect, incidental, special, or consequential damages arising out of this Agreement, except for damages arising from willful misconduct or gross negligence.</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
-        <is>
-          <t>Neither party shall be liable for any indirect, incidental, special, or consequential damages arising out of this Agreement, except for damages arising from willful misconduct or gross negligence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>Specify the governing law to allow for flexibility in jurisdiction.</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>This flexibility can help in case of disputes, allowing for a more favorable legal environment for both parties.</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>Specify the governing law to allow for flexibility in jurisdiction.</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>This Agreement shall be governed by the laws of the State of California or any other mutually agreed jurisdiction.</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>This Agreement shall be governed by the laws of the State of California or any other mutually agreed jurisdiction.</t>
+          <t>Upon termination, each party shall return or destroy all Confidential Information received from the other party, and provide written confirmation of such return or destruction.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
modified:   clauseguard/api/review.py 	modified:   sample_review_export.xlsx
</commit_message>
<xml_diff>
--- a/sample_review_export.xlsx
+++ b/sample_review_export.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,21 +28,25 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
     </font>
     <font>
       <b val="1"/>
-      <sz val="14"/>
+      <color rgb="00C00000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -61,17 +65,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00F3F6FA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -94,11 +93,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -106,7 +103,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -474,21 +471,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ENTERPRISE COMPLIANCE RISK ASSESSMENT REPORT</t>
+          <t>DATA PRIVACY &amp; EXPORT CONTROL COMPLIANCE REVIEW REPORT</t>
         </is>
       </c>
     </row>
@@ -512,308 +512,180 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-16T19:31:14.001300+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Detailed Compliance Findings Table</t>
+          <t>2026-06-17T10:41:06.296493+00:00</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Final Decision</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>CONDITIONAL PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Export Control</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Not Triggered</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Applicable Jurisdictions</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Clause / Section</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Risk Identified</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Risk Level</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Regulation</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Recommended Redline / Mitigation</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>sec. Article 15 - Right of access by the data subject · clause GDPR_Article_15</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>The contract does not address data subject rights such as access and rectification, which are essential under data protection regulations.</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Data Subject Rights - Access/Rectification</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Include clauses in the contract that explicitly address data subject rights, including access and rectification rights as per applicable data protection laws.</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Include clauses in the contract that explicitly address data subject rights, including access and rectification rights as per applicable data protection laws.</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Privacy Jurisdictions:</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>EU</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>sec. Article 15 - Right of access by the data subject · clause GDPR_Article_15</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>The contract does not include provisions for data subject rights such as access and rectification, which are required under GDPR.</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>Data Subject Rights</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>Include clauses that explicitly address data subject rights, including access and rectification rights as per applicable data protection laws.</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Include a clause stating: 'The Parties acknowledge the data subject's rights to access, rectify, and erase their personal data as required by applicable data protection laws.'</t>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Detailed Compliance Findings</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>sec. Article 15 - Right of access by the data subject · clause GDPR_Article_15</t>
+          <t>Issue ID</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Lack of provisions for data subject rights such as access and rectification.</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>high</t>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Clause / Section</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Data Subject Rights</t>
+          <t>Jurisdiction(s)</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Include clauses that explicitly address data subject rights, including access and rectification rights as per applicable data protection laws.</t>
+          <t>Finding</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Include clauses that explicitly address data subject rights, including access and rectification rights as per applicable data protection laws.</t>
+          <t>Risk Level</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Applicable Laws</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Recommended Redline / Mitigation</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Fallback Position</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>p. 1 · sec. GDPR Article 6 · clause GDPR-6</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>The clause mandates compliance with applicable data protection laws, aligning with GDPR requirements.</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Data Protection</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>Ensures that both parties adhere to data protection laws, reducing legal risks.</t>
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>PRIV-001</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>PRIVACY</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>"6.1 Both parties shall comply with applicable data protection laws with respect …"</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>The contract partially addresses the legal basis for processing personal data, but lacks explicit details on the specific legal basis as outlined in GDPR Article 6.
+Evidence status: PARTIALLY_PRESENT. Applicability: The contract includes a section on Data Protection that mentions compliance with applicable data protection laws, indicating personal-data processing obligations. Adequacy: The contract mentions compliance with applicable data protection laws, but does not explicitly state the legal basis for processing personal data as required by Article 6 of the GDPR. Therefore, it partially satisfies the legal obligation.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Consider adding specific provisions for data subject rights, including access and rectification.</t>
-        </is>
-      </c>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Include explicit references to the legal basis for processing personal data as outlined in Article 6 of the GDPR, such as consent or necessity for contract performance.</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>p. 1 · sec. GDPR Article 7 · clause GDPR_Article_7</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>This clause requires prior written consent for disclosing confidential information, aligning with GDPR consent management principles.</t>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>PRIV-012</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>PRIVACY</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Confidentiality</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Protects confidential information from unauthorized disclosure, reducing potential liability.</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Protects confidential information from unauthorized disclosure, reducing potential liability.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>p. 1 · sec. GDPR Article 5 · clause GDPR_Article_5</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>This clause mandates the return or destruction of confidential information upon termination, aligning with GDPR requirements.</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>Data Retention</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>Ensures compliance with data retention and deletion requirements, reducing legal exposure.</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Ensures compliance with data retention and deletion requirements, reducing legal exposure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>p. 1 · sec. GDPR Article 32 · clause GDPR_Article_32</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>This clause requires the implementation of reasonable security measures, aligning with GDPR security requirements.</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Data Protection</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Enhances data protection, reducing the risk of data breaches.</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Enhances data protection, reducing the risk of data breaches.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>sec. Article 15 - Right of access by the data subject · clause GDPR_Article_15</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>This addition will ensure that the contract complies with GDPR requirements regarding data subject rights, reducing legal risks.</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>Ensure compliance with GDPR regarding data subject rights.</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>Include a clause stating: 'The Parties acknowledge the data subject's rights to access, rectify, and erase their personal data as required by applicable data protection laws.'</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Include a clause stating: 'The Parties acknowledge the data subject's rights to access, rectify, and erase their personal data as required by applicable data protection laws.'</t>
-        </is>
-      </c>
+          <t>"1.2 The receiving party shall not disclose Confidential Information to any third…"</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr"/>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>The control is partially satisfied as the contract provides some transparency regarding confidentiality but lacks comprehensive disclosures required under GDPR.
+Evidence status: PARTIALLY_PRESENT. Applicability: The contract includes a section on Data Protection that mentions compliance with applicable data protection laws, indicating personal-data processing obligations, which triggers the need for transparency and disclosures regarding personal data. Adequacy: The contract includes a confidentiality clause that addresses the need for consent before disclosing confidential information, which is relevant to transparency. However, it lacks specific details on the disclosures required under GDPR, such as the purposes of processing and the rights of data subjects, making it materially weaker than the legal obligation.</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr"/>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Enhance the contract by including specific disclosures about the purposes of data processing, the rights of data subjects, and any other relevant transparency obligations under GDPR.</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>